<commit_message>
Document TIX/KILROY/CONNECTIONS' slow-load behavior in sites.xlsx
No code change -- the URL templates are correct as shipped. Investigated
a report of TIX showing blank/stuck on a phone, which led down a false
trail (a missing searchId/searchRequestId session parameter) before
confirming with longer waits (and the user's own real-Chrome retest)
that these sites just take 5-30s to resolve real search results and
the "session id" tix.nl ends up with in the address bar is something it
appends itself once results are ready, not something we need to supply.
Documenting this so nobody re-diagnoses the same false trail later.
</commit_message>
<xml_diff>
--- a/data/sites.xlsx
+++ b/data/sites.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>已根据实测 URL 配置，未做二次验证（没有反复测试是否每次都稳定生效），建议首次使用留意一下结果是否正确。</t>
+          <t>已根据实测 URL 配置。注意：打开后网站需要几秒到二十几秒查询真实结果（查询完成后网站会自己在地址栏加一个 searchId，不用我们提供），刚打开时页面可能显示筛选栏但结果区域是加载动画，属于正常现象，耐心等一下就好，不是链接错了。</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>实测 URL 里还带了一个 searchRequestId（随机会话 ID），这里的模板里去掉了，因为没法预先构造出有效值。如果打开后页面提示错误或空结果，说明这个网站强制要求这个 ID，只能退回"打开首页手动搜索"（把这一行的模板列清空即可）。日期格式和其他网站不一样，是"日.月.年"，模板已用 {dateDDMMYYYY} 占位符处理。</t>
+          <t>已根据实测 URL 配置。同 TIX，打开后需要等待（实测约 20-30 秒）才会出真实结果，等待期间会显示"Searching for flights..."，属于正常现象。日期格式和其他网站不一样，是"日.月.年"，模板已用 {dateDDMMYYYY} 占位符处理。</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>实测 URL 里 from/to 参数带了 A-（具体机场）或 C-（多机场城市，如北京 BJS、东京 TYO）前缀，模板用 {originWithPrefix}/{destinationWithPrefix} 占位符自动处理（哪些代码算"多机场城市"在 lib/buildSearchUrl.js 的 MULTI_AIRPORT_CITY_CODES 里，可以按需编辑）。还去掉了一个 journeyUid 随机 ID，没做二次验证，建议首次使用留意结果是否正确。</t>
+          <t>已根据实测 URL 配置，from/to 参数带了 A-（具体机场）或 C-（多机场城市，如北京 BJS、东京 TYO）前缀，模板用 {originWithPrefix}/{destinationWithPrefix} 占位符自动处理（哪些代码算"多机场城市"在 lib/buildSearchUrl.js 的 MULTI_AIRPORT_CITY_CODES 里，可以按需编辑）。同样可能需要等待才出结果，如果打开后长时间只显示"欢迎搜索"的提示而不是结果，先多等一会/刷新一次再判断是否有问题。</t>
         </is>
       </c>
     </row>

</xml_diff>